<commit_message>
edit charts + hamburger
</commit_message>
<xml_diff>
--- a/outputs/feb3/MAIN_feb3.xlsx
+++ b/outputs/feb3/MAIN_feb3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edreiyu/Documents/Projects/vat_burden_analysis/outputs/feb3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65FEEF43-32D7-2349-A360-449AFF82094F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BD7F2A-D576-F649-BF2A-DE4B185A3500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5540" yWindow="2120" windowWidth="27880" windowHeight="17440" activeTab="4" xr2:uid="{30613F82-6F92-CA4A-972E-4B9F4D12BC37}"/>
+    <workbookView xWindow="5080" yWindow="1360" windowWidth="27880" windowHeight="17440" activeTab="2" xr2:uid="{30613F82-6F92-CA4A-972E-4B9F4D12BC37}"/>
   </bookViews>
   <sheets>
     <sheet name="main_summary" sheetId="8" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="149">
   <si>
     <t>NPCINC</t>
   </si>
@@ -5064,14 +5064,18 @@
   <cols>
     <col min="1" max="1" width="27.83203125" style="7" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1640625" customWidth="1"/>
-    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
     <col min="7" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="16" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="18" max="31" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6122,7 +6126,7 @@
     </row>
     <row r="12" spans="1:31">
       <c r="A12" s="20" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B12" s="3">
         <f>SUM(B2:B11)</f>
@@ -6189,12 +6193,69 @@
         <v>506482095007.60693</v>
       </c>
     </row>
-    <row r="14" spans="1:31">
-      <c r="A14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="2">
-        <v>27479695.00677811</v>
+    <row r="13" spans="1:31">
+      <c r="A13" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="2">
+        <f>C12*12</f>
+        <v>2506710392742.2578</v>
+      </c>
+      <c r="D13" s="2">
+        <f t="shared" ref="D13:Q13" si="1">D12*12</f>
+        <v>100389142139.08801</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="1"/>
+        <v>136827721913.48099</v>
+      </c>
+      <c r="F13" s="2">
+        <f t="shared" si="1"/>
+        <v>786108666022.97705</v>
+      </c>
+      <c r="G13" s="2">
+        <f t="shared" si="1"/>
+        <v>219258572685.33044</v>
+      </c>
+      <c r="H13" s="2">
+        <f t="shared" si="1"/>
+        <v>209662291517.31628</v>
+      </c>
+      <c r="I13" s="2">
+        <f t="shared" si="1"/>
+        <v>538821272046.04932</v>
+      </c>
+      <c r="J13" s="2">
+        <f t="shared" si="1"/>
+        <v>289983936696.05524</v>
+      </c>
+      <c r="K13" s="2">
+        <f t="shared" si="1"/>
+        <v>60672066322.912491</v>
+      </c>
+      <c r="L13" s="2">
+        <f t="shared" si="1"/>
+        <v>234069580099.78171</v>
+      </c>
+      <c r="M13" s="2">
+        <f t="shared" si="1"/>
+        <v>401795823333.00537</v>
+      </c>
+      <c r="N13" s="2">
+        <f t="shared" si="1"/>
+        <v>193691709260.89212</v>
+      </c>
+      <c r="O13" s="2">
+        <f t="shared" si="1"/>
+        <v>262297106646.7597</v>
+      </c>
+      <c r="P13" s="2">
+        <f t="shared" si="1"/>
+        <v>137496858665.36877</v>
+      </c>
+      <c r="Q13" s="2">
+        <f t="shared" si="1"/>
+        <v>6077785140091.2832</v>
       </c>
     </row>
     <row r="15" spans="1:31">
@@ -6202,8 +6263,12 @@
       <c r="B15" s="2"/>
     </row>
     <row r="16" spans="1:31">
-      <c r="A16"/>
-      <c r="B16" s="2"/>
+      <c r="A16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="2">
+        <v>27479695.00677811</v>
+      </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
@@ -6241,7 +6306,7 @@
         <v>141408880112.64801</v>
       </c>
       <c r="E19" s="37">
-        <f t="shared" ref="E19" si="1">D19/D$33</f>
+        <f t="shared" ref="E19" si="2">D19/D$33</f>
         <v>0.27919818194268886</v>
       </c>
       <c r="F19" s="6">
@@ -6257,18 +6322,18 @@
         <v>8365761844.9240017</v>
       </c>
       <c r="C20" s="37">
-        <f t="shared" ref="C20:E33" si="2">B20/B$33</f>
+        <f t="shared" ref="C20:E33" si="3">B20/B$33</f>
         <v>1.6517389118757209E-2</v>
       </c>
       <c r="D20" s="35">
         <v>0</v>
       </c>
       <c r="E20" s="37">
-        <f t="shared" ref="E20" si="3">D20/D$33</f>
+        <f t="shared" ref="E20" si="4">D20/D$33</f>
         <v>0</v>
       </c>
       <c r="F20" s="6">
-        <f t="shared" ref="F20:F33" si="4">D20/B20</f>
+        <f t="shared" ref="F20:F33" si="5">D20/B20</f>
         <v>0</v>
       </c>
     </row>
@@ -6280,18 +6345,18 @@
         <v>11402310159.456749</v>
       </c>
       <c r="C21" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.2512760612565179E-2</v>
       </c>
       <c r="D21" s="35">
         <v>0</v>
       </c>
       <c r="E21" s="37">
-        <f t="shared" ref="E21" si="5">D21/D$33</f>
+        <f t="shared" ref="E21" si="6">D21/D$33</f>
         <v>0</v>
       </c>
       <c r="F21" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -6303,18 +6368,18 @@
         <v>65509055501.914749</v>
       </c>
       <c r="C22" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.12934130573940794</v>
       </c>
       <c r="D22" s="36">
         <v>17708984981.132751</v>
       </c>
       <c r="E22" s="37">
-        <f t="shared" ref="E22" si="6">D22/D$33</f>
+        <f t="shared" ref="E22" si="7">D22/D$33</f>
         <v>3.4964681191477824E-2</v>
       </c>
       <c r="F22" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.27032880943635557</v>
       </c>
     </row>
@@ -6326,18 +6391,18 @@
         <v>18271547723.777538</v>
       </c>
       <c r="C23" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.6075407016121892E-2</v>
       </c>
       <c r="D23" s="36">
         <v>4234047000.5916023</v>
       </c>
       <c r="E23" s="37">
-        <f t="shared" ref="E23" si="7">D23/D$33</f>
+        <f t="shared" ref="E23" si="8">D23/D$33</f>
         <v>8.3597170409903873E-3</v>
       </c>
       <c r="F23" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.23172897362611805</v>
       </c>
     </row>
@@ -6349,18 +6414,18 @@
         <v>17471857626.443024</v>
       </c>
       <c r="C24" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.4496496122297493E-2</v>
       </c>
       <c r="D24" s="36">
         <v>9674287392.363163</v>
       </c>
       <c r="E24" s="37">
-        <f t="shared" ref="E24" si="8">D24/D$33</f>
+        <f t="shared" ref="E24" si="9">D24/D$33</f>
         <v>1.9100946485024053E-2</v>
       </c>
       <c r="F24" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.55370685814892862</v>
       </c>
     </row>
@@ -6372,18 +6437,18 @@
         <v>44901772670.504112</v>
       </c>
       <c r="C25" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>8.8654215248872181E-2</v>
       </c>
       <c r="D25" s="36">
         <v>16613633534.112116</v>
       </c>
       <c r="E25" s="37">
-        <f t="shared" ref="E25" si="9">D25/D$33</f>
+        <f t="shared" ref="E25" si="10">D25/D$33</f>
         <v>3.2802015506318345E-2</v>
       </c>
       <c r="F25" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.36999950215830968</v>
       </c>
     </row>
@@ -6395,18 +6460,18 @@
         <v>24165328058.004604</v>
       </c>
       <c r="C26" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.7712107291061616E-2</v>
       </c>
       <c r="D26" s="36">
         <v>0</v>
       </c>
       <c r="E26" s="37">
-        <f t="shared" ref="E26" si="10">D26/D$33</f>
+        <f t="shared" ref="E26" si="11">D26/D$33</f>
         <v>0</v>
       </c>
       <c r="F26" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -6418,18 +6483,18 @@
         <v>5056005526.9093742</v>
       </c>
       <c r="C27" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.9825947980124296E-3</v>
       </c>
       <c r="D27" s="36">
         <v>456625856.80066192</v>
       </c>
       <c r="E27" s="37">
-        <f t="shared" ref="E27" si="11">D27/D$33</f>
+        <f t="shared" ref="E27" si="12">D27/D$33</f>
         <v>9.015636708614626E-4</v>
       </c>
       <c r="F27" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>9.0313559660957748E-2</v>
       </c>
     </row>
@@ -6441,18 +6506,18 @@
         <v>19505798341.648476</v>
       </c>
       <c r="C28" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.8512315704576909E-2</v>
       </c>
       <c r="D28" s="36">
         <v>18490627235.181778</v>
       </c>
       <c r="E28" s="37">
-        <f t="shared" ref="E28" si="12">D28/D$33</f>
+        <f t="shared" ref="E28" si="13">D28/D$33</f>
         <v>3.6507958361102724E-2</v>
       </c>
       <c r="F28" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.94795541875878409</v>
       </c>
     </row>
@@ -6464,18 +6529,18 @@
         <v>33482985277.75045</v>
       </c>
       <c r="C29" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.6108921929900727E-2</v>
       </c>
       <c r="D29" s="36">
         <v>0</v>
       </c>
       <c r="E29" s="37">
-        <f t="shared" ref="E29" si="13">D29/D$33</f>
+        <f t="shared" ref="E29" si="14">D29/D$33</f>
         <v>0</v>
       </c>
       <c r="F29" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -6487,18 +6552,18 @@
         <v>16140975771.741011</v>
       </c>
       <c r="C30" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1868798385653867E-2</v>
       </c>
       <c r="D30" s="36">
         <v>14876516517.106092</v>
       </c>
       <c r="E30" s="37">
-        <f t="shared" ref="E30" si="14">D30/D$33</f>
+        <f t="shared" ref="E30" si="15">D30/D$33</f>
         <v>2.9372245660298547E-2</v>
       </c>
       <c r="F30" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.92166153567687747</v>
       </c>
     </row>
@@ -6510,18 +6575,18 @@
         <v>21858092220.563309</v>
       </c>
       <c r="C31" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.3156692874276273E-2</v>
       </c>
       <c r="D31" s="36">
         <v>0</v>
       </c>
       <c r="E31" s="37">
-        <f t="shared" ref="E31" si="15">D31/D$33</f>
+        <f t="shared" ref="E31" si="16">D31/D$33</f>
         <v>0</v>
       </c>
       <c r="F31" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -6533,18 +6598,18 @@
         <v>11458071555.447399</v>
       </c>
       <c r="C32" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.2622856105654256E-2</v>
       </c>
       <c r="D32" s="36">
         <v>0</v>
       </c>
       <c r="E32" s="37">
-        <f t="shared" ref="E32" si="16">D32/D$33</f>
+        <f t="shared" ref="E32" si="17">D32/D$33</f>
         <v>0</v>
       </c>
       <c r="F32" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -6556,18 +6621,18 @@
         <v>506482095007.60693</v>
       </c>
       <c r="C33" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D33" s="36">
         <v>506482095007.60669</v>
       </c>
       <c r="E33" s="37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="F33" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.99999999999999956</v>
       </c>
     </row>

</xml_diff>